<commit_message>
Implemented end-to-end Selenium automation framework
</commit_message>
<xml_diff>
--- a/test_data/Task_15 (1).xlsx
+++ b/test_data/Task_15 (1).xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="13">
   <si>
     <t>TestID</t>
   </si>
@@ -50,6 +50,9 @@
   </si>
   <si>
     <t>jsjnsd</t>
+  </si>
+  <si>
+    <t>Nil</t>
   </si>
 </sst>
 </file>
@@ -135,9 +138,8 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -152,7 +154,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -453,324 +455,316 @@
   <cols>
     <col min="1" max="1" width="16.5703125" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="8" width="16.5703125" customWidth="1"/>
-    <col min="9" max="13" width="16.5703125" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="16.5703125" style="1"/>
+    <col min="3" max="4" width="16.5703125" customWidth="1"/>
+    <col min="5" max="5" width="31.5703125" customWidth="1"/>
+    <col min="6" max="8" width="16.5703125" customWidth="1"/>
+    <col min="9" max="17" width="16.5703125" style="7" customWidth="1"/>
+    <col min="18" max="16384" width="16.5703125" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1"/>
+      <c r="H1" s="7"/>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="3">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="3" t="s">
+      <c r="C2" s="6"/>
+      <c r="D2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="3"/>
-      <c r="H2" s="1"/>
-    </row>
-    <row r="3" spans="1:8" ht="45" customHeight="1">
-      <c r="A3" s="3">
+      <c r="G2" s="2"/>
+      <c r="H2" s="7"/>
+    </row>
+    <row r="3" spans="1:8" ht="15" customHeight="1">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="5" t="s">
+      <c r="C3" s="6"/>
+      <c r="D3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="3"/>
-      <c r="H3" s="1"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="7"/>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="3">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="3" t="s">
+      <c r="C4" s="6"/>
+      <c r="D4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="1"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="7"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="3">
-        <v>4</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="1"/>
+      <c r="A5" s="2"/>
+      <c r="B5" s="5"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="7"/>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="3">
-        <v>5</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="1"/>
+      <c r="A6" s="2"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="7"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="2"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="1"/>
+      <c r="A7" s="1"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="7"/>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
+      <c r="A8" s="7"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
+      <c r="A9" s="7"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
+      <c r="A11" s="7"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="1"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
+      <c r="A12" s="7"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="1"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
+      <c r="A13" s="7"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="1"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
+      <c r="A14" s="7"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="1"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
+      <c r="A15" s="7"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="1"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
+      <c r="A16" s="7"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
+      <c r="A17" s="7"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
     </row>
     <row r="18" spans="1:8">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
+      <c r="A18" s="7"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
     </row>
     <row r="19" spans="1:8">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
+      <c r="A19" s="7"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
     </row>
     <row r="20" spans="1:8">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
+      <c r="A20" s="7"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="7"/>
     </row>
     <row r="21" spans="1:8">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
+      <c r="A21" s="7"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="7"/>
     </row>
     <row r="22" spans="1:8">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
+      <c r="A22" s="7"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
     </row>
     <row r="23" spans="1:8">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
+      <c r="A23" s="7"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="7"/>
     </row>
     <row r="24" spans="1:8">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
+      <c r="A24" s="7"/>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
+      <c r="H24" s="7"/>
     </row>
     <row r="25" spans="1:8">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
+      <c r="A25" s="7"/>
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+      <c r="H25" s="7"/>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
+      <c r="A26" s="7"/>
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="7"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>